<commit_message>
feat: add different-event attribution type
</commit_message>
<xml_diff>
--- a/examples/attribution_eval_candidates_annotate.xlsx
+++ b/examples/attribution_eval_candidates_annotate.xlsx
@@ -771,14 +771,10 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>event-type mismatch</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -1340,7 +1336,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1816,7 +1812,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>entity mismatch</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1937,14 +1933,10 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -2639,7 +2631,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -3123,14 +3115,10 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -4999,14 +4987,10 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>event-type mismatch</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -5229,14 +5213,10 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>event-type mismatch</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -7101,14 +7081,10 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
+          <t>benign illustrative image</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
           <t>benign illustrative image</t>
@@ -8033,7 +8009,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>location mismatch</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -8388,7 +8364,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>event-type mismatch</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -10123,7 +10099,7 @@
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation sqref="L2:L81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Options!$A$2:$A$9</formula1>
+      <formula1>=Options!$A$2:$A$10</formula1>
     </dataValidation>
     <dataValidation sqref="M2:S81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=Options!$C$2:$C$3</formula1>
@@ -10149,7 +10125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -10347,7 +10323,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>context omission</t>
+          <t>different-event mismatch</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
@@ -10366,7 +10342,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>uncertain / evidence insufficient</t>
+          <t>context omission</t>
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
@@ -10377,6 +10353,21 @@
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>uncertain / evidence insufficient</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10389,7 +10380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -10476,17 +10467,24 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>OOC 且整件事都对不上：gold_mismatch_type 选 different-event mismatch，并把多个冲突字段选 Y。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>标完后导回 JSONL：</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>标完后导回 JSONL：</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>python scripts\eval\import_attribution_xlsx.py --xlsx examples\attribution_eval_candidates_annotate.xlsx --output examples\attribution_eval_set.jsonl</t>
         </is>

</xml_diff>